<commit_message>
added sfsac download option and links to bulk mdl
</commit_message>
<xml_diff>
--- a/input_multiple_results.xlsx
+++ b/input_multiple_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -439,16 +439,6 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>local_path</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
           <t>message</t>
         </is>
       </c>
@@ -472,17 +462,7 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>D:\Documents\Profesh\Forward Edge AI\Treasury AI\single-finding-fix\mdl-backend-demo\outputs\MDL-City_of_Carson-952513547-2023.docx</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>http://localhost:8000/local/mdl/2023/MDL-City_of_Carson-952513547-2023.docx</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -503,17 +483,7 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>D:\Documents\Profesh\Forward Edge AI\Treasury AI\single-finding-fix\mdl-backend-demo\outputs\MDL-City_of_West_Haven_CT-066002126-2023.docx</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>http://localhost:8000/local/mdl/2023/MDL-City_of_West_Haven_CT-066002126-2023.docx</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -534,17 +504,7 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>D:\Documents\Profesh\Forward Edge AI\Treasury AI\single-finding-fix\mdl-backend-demo\outputs\MDL-COBB_COUNTY_GOVERNMENT-586000804-2022.docx</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>http://localhost:8000/local/mdl/2022/MDL-COBB_COUNTY_GOVERNMENT-586000804-2022.docx</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -565,17 +525,7 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>D:\Documents\Profesh\Forward Edge AI\Treasury AI\single-finding-fix\mdl-backend-demo\outputs\MDL-SANTA ROSA BAND_OF_CAHUILLA_INDIANS-330884665-2022.docx</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>http://localhost:8000/local/mdl/2022/MDL-SANTA_ROSA_BAND_OF_CAHUILLA_INDIANS-330884665-2022.docx</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -596,17 +546,7 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>D:\Documents\Profesh\Forward Edge AI\Treasury AI\single-finding-fix\mdl-backend-demo\outputs\MDL-TOWN_OF_ELKTON_VIRGINIA-546001261-2024.docx</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>http://localhost:8000/local/mdl/2024/MDL-TOWN_OF_ELKTON_VIRGINIA-546001261-2024.docx</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -627,17 +567,28 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>D:\Documents\Profesh\Forward Edge AI\Treasury AI\single-finding-fix\mdl-backend-demo\outputs\MDL-TOWN_OF_RUTLAND_MASSACHUSETTS-046001287-2023.docx</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>http://localhost:8000/local/mdl/2023/MDL-TOWN_OF_RUTLAND_MASSACHUSETTS-046001287-2023.docx</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>311334820</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>State of Ohio</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>